<commit_message>
EV2: resultados de la prueba de estrés en AWS
- docs/pruebas/estres/aws: Locust 10 → 100 usuarios contra EC2 t3.small y monitor de CPU/memoria
- Matriz regenerada: 138/138 pruebas aprobadas, hojas Estrés y Umbrales con datos de AWS
- README: tabla de resultados, degradación observada y límite seguro

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pruebas/matriz_pruebas_sgr_ev2.xlsx
+++ b/docs/pruebas/matriz_pruebas_sgr_ev2.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz funcional" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pruebas automatizadas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estrés" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Umbrales" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendientes y simulados" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Matriz funcional" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pruebas automatizadas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Estrés" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Umbrales" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pendientes y simulados" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz funcional'!$A$4:$K$46</definedName>
@@ -52,7 +52,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +72,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF4E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE7E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -101,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,6 +123,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -511,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SGR La Serena · EV2 · 42 casos · 42 aprobados · base de datos de prueba: mysql · generado 16-10-2026 20:43</t>
+          <t>SGR La Serena · EV2 · 42 casos · 42 aprobados · base de datos de prueba: sqlite3 · generado 17-10-2026 12:02</t>
         </is>
       </c>
     </row>
@@ -625,7 +633,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -682,7 +690,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -739,7 +747,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -796,7 +804,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -853,7 +861,7 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -910,7 +918,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -967,7 +975,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1032,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1089,7 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1146,7 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1203,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1260,7 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1317,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1374,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1431,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1488,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1545,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1602,7 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1659,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1716,7 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1773,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1822,7 +1830,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1887,7 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1944,7 @@
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -1993,7 +2001,7 @@
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2058,7 @@
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2115,7 @@
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2172,7 @@
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2229,7 @@
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2286,7 @@
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2343,7 @@
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2400,7 @@
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2457,7 @@
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2514,7 @@
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2571,7 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2628,7 @@
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2685,7 @@
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2742,7 @@
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2799,7 @@
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2856,7 @@
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2913,7 @@
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2970,7 @@
       </c>
       <c r="K46" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3087,7 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
     </row>
@@ -3115,7 +3123,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
     </row>
@@ -3151,7 +3159,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
@@ -3187,7 +3195,7 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="H8" s="4" t="inlineStr"/>
     </row>
@@ -3223,7 +3231,7 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
@@ -3259,7 +3267,7 @@
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4" t="inlineStr"/>
     </row>
@@ -3295,7 +3303,7 @@
         </is>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
@@ -3331,7 +3339,7 @@
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
     </row>
@@ -3367,7 +3375,7 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="H13" s="4" t="inlineStr"/>
     </row>
@@ -3403,7 +3411,7 @@
         </is>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H14" s="4" t="inlineStr"/>
     </row>
@@ -3439,7 +3447,7 @@
         </is>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H15" s="4" t="inlineStr"/>
     </row>
@@ -3475,7 +3483,7 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
     </row>
@@ -3511,7 +3519,7 @@
         </is>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="H17" s="4" t="inlineStr"/>
     </row>
@@ -3583,7 +3591,7 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
     </row>
@@ -3619,7 +3627,7 @@
         </is>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.99</v>
+        <v>0.19</v>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
     </row>
@@ -3655,7 +3663,7 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H21" s="4" t="inlineStr"/>
     </row>
@@ -3691,7 +3699,7 @@
         </is>
       </c>
       <c r="G22" s="4" t="n">
-        <v>0.12</v>
+        <v>0.03</v>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
     </row>
@@ -3727,7 +3735,7 @@
         </is>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
     </row>
@@ -3763,7 +3771,7 @@
         </is>
       </c>
       <c r="G24" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
     </row>
@@ -3799,7 +3807,7 @@
         </is>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
     </row>
@@ -3835,7 +3843,7 @@
         </is>
       </c>
       <c r="G26" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
     </row>
@@ -3871,7 +3879,7 @@
         </is>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
     </row>
@@ -3907,7 +3915,7 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
     </row>
@@ -3943,7 +3951,7 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0.12</v>
+        <v>0.02</v>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
     </row>
@@ -3979,7 +3987,7 @@
         </is>
       </c>
       <c r="G30" s="4" t="n">
-        <v>0.08</v>
+        <v>0.01</v>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
     </row>
@@ -4015,7 +4023,7 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
     </row>
@@ -4051,7 +4059,7 @@
         </is>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
     </row>
@@ -4087,7 +4095,7 @@
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
     </row>
@@ -4123,7 +4131,7 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
     </row>
@@ -4159,7 +4167,7 @@
         </is>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
     </row>
@@ -4195,7 +4203,7 @@
         </is>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
     </row>
@@ -4231,7 +4239,7 @@
         </is>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
     </row>
@@ -4267,7 +4275,7 @@
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
     </row>
@@ -4303,7 +4311,7 @@
         </is>
       </c>
       <c r="G39" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
     </row>
@@ -4339,7 +4347,7 @@
         </is>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
     </row>
@@ -4375,7 +4383,7 @@
         </is>
       </c>
       <c r="G41" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
     </row>
@@ -4411,7 +4419,7 @@
         </is>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
     </row>
@@ -4447,7 +4455,7 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
     </row>
@@ -4483,7 +4491,7 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
     </row>
@@ -4519,7 +4527,7 @@
         </is>
       </c>
       <c r="G45" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
     </row>
@@ -4555,7 +4563,7 @@
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
     </row>
@@ -4591,7 +4599,7 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
     </row>
@@ -4627,7 +4635,7 @@
         </is>
       </c>
       <c r="G48" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="H48" s="4" t="inlineStr"/>
     </row>
@@ -4663,7 +4671,7 @@
         </is>
       </c>
       <c r="G49" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
     </row>
@@ -4699,7 +4707,7 @@
         </is>
       </c>
       <c r="G50" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H50" s="4" t="inlineStr"/>
     </row>
@@ -4735,7 +4743,7 @@
         </is>
       </c>
       <c r="G51" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="H51" s="4" t="inlineStr"/>
     </row>
@@ -4771,7 +4779,7 @@
         </is>
       </c>
       <c r="G52" s="4" t="n">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="H52" s="4" t="inlineStr"/>
     </row>
@@ -4807,7 +4815,7 @@
         </is>
       </c>
       <c r="G53" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H53" s="4" t="inlineStr"/>
     </row>
@@ -4843,7 +4851,7 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H54" s="4" t="inlineStr"/>
     </row>
@@ -4879,7 +4887,7 @@
         </is>
       </c>
       <c r="G55" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H55" s="4" t="inlineStr"/>
     </row>
@@ -4915,7 +4923,7 @@
         </is>
       </c>
       <c r="G56" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H56" s="4" t="inlineStr"/>
     </row>
@@ -4951,7 +4959,7 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H57" s="4" t="inlineStr"/>
     </row>
@@ -4987,7 +4995,7 @@
         </is>
       </c>
       <c r="G58" s="4" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="H58" s="4" t="inlineStr"/>
     </row>
@@ -5023,7 +5031,7 @@
         </is>
       </c>
       <c r="G59" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="H59" s="4" t="inlineStr"/>
     </row>
@@ -5059,7 +5067,7 @@
         </is>
       </c>
       <c r="G60" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="H60" s="4" t="inlineStr"/>
     </row>
@@ -5095,7 +5103,7 @@
         </is>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="H61" s="4" t="inlineStr"/>
     </row>
@@ -5131,7 +5139,7 @@
         </is>
       </c>
       <c r="G62" s="4" t="n">
-        <v>0.18</v>
+        <v>0.02</v>
       </c>
       <c r="H62" s="4" t="inlineStr"/>
     </row>
@@ -5167,7 +5175,7 @@
         </is>
       </c>
       <c r="G63" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H63" s="4" t="inlineStr"/>
     </row>
@@ -5203,7 +5211,7 @@
         </is>
       </c>
       <c r="G64" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H64" s="4" t="inlineStr"/>
     </row>
@@ -5239,7 +5247,7 @@
         </is>
       </c>
       <c r="G65" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H65" s="4" t="inlineStr"/>
     </row>
@@ -5275,7 +5283,7 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H66" s="4" t="inlineStr"/>
     </row>
@@ -5311,7 +5319,7 @@
         </is>
       </c>
       <c r="G67" s="4" t="n">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="H67" s="4" t="inlineStr"/>
     </row>
@@ -5347,7 +5355,7 @@
         </is>
       </c>
       <c r="G68" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H68" s="4" t="inlineStr"/>
     </row>
@@ -5383,7 +5391,7 @@
         </is>
       </c>
       <c r="G69" s="4" t="n">
-        <v>0.13</v>
+        <v>0.02</v>
       </c>
       <c r="H69" s="4" t="inlineStr"/>
     </row>
@@ -5419,7 +5427,7 @@
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H70" s="4" t="inlineStr"/>
     </row>
@@ -5455,7 +5463,7 @@
         </is>
       </c>
       <c r="G71" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H71" s="4" t="inlineStr"/>
     </row>
@@ -5491,7 +5499,7 @@
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H72" s="4" t="inlineStr"/>
     </row>
@@ -5527,7 +5535,7 @@
         </is>
       </c>
       <c r="G73" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H73" s="4" t="inlineStr"/>
     </row>
@@ -5563,7 +5571,7 @@
         </is>
       </c>
       <c r="G74" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="H74" s="4" t="inlineStr"/>
     </row>
@@ -5599,7 +5607,7 @@
         </is>
       </c>
       <c r="G75" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H75" s="4" t="inlineStr"/>
     </row>
@@ -5635,7 +5643,7 @@
         </is>
       </c>
       <c r="G76" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H76" s="4" t="inlineStr"/>
     </row>
@@ -5671,7 +5679,7 @@
         </is>
       </c>
       <c r="G77" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H77" s="4" t="inlineStr"/>
     </row>
@@ -5707,7 +5715,7 @@
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H78" s="4" t="inlineStr"/>
     </row>
@@ -5743,7 +5751,7 @@
         </is>
       </c>
       <c r="G79" s="4" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="H79" s="4" t="inlineStr"/>
     </row>
@@ -5779,7 +5787,7 @@
         </is>
       </c>
       <c r="G80" s="4" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="H80" s="4" t="inlineStr"/>
     </row>
@@ -5851,7 +5859,7 @@
         </is>
       </c>
       <c r="G82" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H82" s="4" t="inlineStr"/>
     </row>
@@ -5887,7 +5895,7 @@
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="H83" s="4" t="inlineStr"/>
     </row>
@@ -5923,7 +5931,7 @@
         </is>
       </c>
       <c r="G84" s="4" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="H84" s="4" t="inlineStr"/>
     </row>
@@ -5959,7 +5967,7 @@
         </is>
       </c>
       <c r="G85" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H85" s="4" t="inlineStr"/>
     </row>
@@ -5995,7 +6003,7 @@
         </is>
       </c>
       <c r="G86" s="4" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="H86" s="4" t="inlineStr"/>
     </row>
@@ -6031,7 +6039,7 @@
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H87" s="4" t="inlineStr"/>
     </row>
@@ -6067,7 +6075,7 @@
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H88" s="4" t="inlineStr"/>
     </row>
@@ -6103,7 +6111,7 @@
         </is>
       </c>
       <c r="G89" s="4" t="n">
-        <v>0.04</v>
+        <v>1.31</v>
       </c>
       <c r="H89" s="4" t="inlineStr"/>
     </row>
@@ -6139,7 +6147,7 @@
         </is>
       </c>
       <c r="G90" s="4" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="H90" s="4" t="inlineStr"/>
     </row>
@@ -6175,7 +6183,7 @@
         </is>
       </c>
       <c r="G91" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H91" s="4" t="inlineStr"/>
     </row>
@@ -6211,7 +6219,7 @@
         </is>
       </c>
       <c r="G92" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H92" s="4" t="inlineStr"/>
     </row>
@@ -6247,7 +6255,7 @@
         </is>
       </c>
       <c r="G93" s="4" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="H93" s="4" t="inlineStr"/>
     </row>
@@ -6283,7 +6291,7 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="H94" s="4" t="inlineStr"/>
     </row>
@@ -6319,7 +6327,7 @@
         </is>
       </c>
       <c r="G95" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H95" s="4" t="inlineStr"/>
     </row>
@@ -6355,7 +6363,7 @@
         </is>
       </c>
       <c r="G96" s="4" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="H96" s="4" t="inlineStr"/>
     </row>
@@ -6391,7 +6399,7 @@
         </is>
       </c>
       <c r="G97" s="4" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="H97" s="4" t="inlineStr"/>
     </row>
@@ -6427,7 +6435,7 @@
         </is>
       </c>
       <c r="G98" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H98" s="4" t="inlineStr"/>
     </row>
@@ -6463,7 +6471,7 @@
         </is>
       </c>
       <c r="G99" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H99" s="4" t="inlineStr"/>
     </row>
@@ -6499,7 +6507,7 @@
         </is>
       </c>
       <c r="G100" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H100" s="4" t="inlineStr"/>
     </row>
@@ -6535,7 +6543,7 @@
         </is>
       </c>
       <c r="G101" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H101" s="4" t="inlineStr"/>
     </row>
@@ -6571,7 +6579,7 @@
         </is>
       </c>
       <c r="G102" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H102" s="4" t="inlineStr"/>
     </row>
@@ -6607,7 +6615,7 @@
         </is>
       </c>
       <c r="G103" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="H103" s="4" t="inlineStr"/>
     </row>
@@ -6643,7 +6651,7 @@
         </is>
       </c>
       <c r="G104" s="4" t="n">
-        <v>0.08</v>
+        <v>0.01</v>
       </c>
       <c r="H104" s="4" t="inlineStr"/>
     </row>
@@ -6679,7 +6687,7 @@
         </is>
       </c>
       <c r="G105" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="H105" s="4" t="inlineStr"/>
     </row>
@@ -6715,7 +6723,7 @@
         </is>
       </c>
       <c r="G106" s="4" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="H106" s="4" t="inlineStr"/>
     </row>
@@ -6751,7 +6759,7 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="H107" s="4" t="inlineStr"/>
     </row>
@@ -6787,7 +6795,7 @@
         </is>
       </c>
       <c r="G108" s="4" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="H108" s="4" t="inlineStr"/>
     </row>
@@ -6823,7 +6831,7 @@
         </is>
       </c>
       <c r="G109" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H109" s="4" t="inlineStr"/>
     </row>
@@ -6859,7 +6867,7 @@
         </is>
       </c>
       <c r="G110" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="H110" s="4" t="inlineStr"/>
     </row>
@@ -6895,7 +6903,7 @@
         </is>
       </c>
       <c r="G111" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H111" s="4" t="inlineStr"/>
     </row>
@@ -6931,7 +6939,7 @@
         </is>
       </c>
       <c r="G112" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H112" s="4" t="inlineStr"/>
     </row>
@@ -6967,7 +6975,7 @@
         </is>
       </c>
       <c r="G113" s="4" t="n">
-        <v>0.08</v>
+        <v>0.01</v>
       </c>
       <c r="H113" s="4" t="inlineStr"/>
     </row>
@@ -7003,7 +7011,7 @@
         </is>
       </c>
       <c r="G114" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H114" s="4" t="inlineStr"/>
     </row>
@@ -7039,7 +7047,7 @@
         </is>
       </c>
       <c r="G115" s="4" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="H115" s="4" t="inlineStr"/>
     </row>
@@ -7075,7 +7083,7 @@
         </is>
       </c>
       <c r="G116" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="H116" s="4" t="inlineStr"/>
     </row>
@@ -7111,7 +7119,7 @@
         </is>
       </c>
       <c r="G117" s="4" t="n">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="H117" s="4" t="inlineStr"/>
     </row>
@@ -7147,7 +7155,7 @@
         </is>
       </c>
       <c r="G118" s="4" t="n">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="H118" s="4" t="inlineStr"/>
     </row>
@@ -7183,7 +7191,7 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="H119" s="4" t="inlineStr"/>
     </row>
@@ -7219,7 +7227,7 @@
         </is>
       </c>
       <c r="G120" s="4" t="n">
-        <v>0.08</v>
+        <v>0.01</v>
       </c>
       <c r="H120" s="4" t="inlineStr"/>
     </row>
@@ -7255,7 +7263,7 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H121" s="4" t="inlineStr"/>
     </row>
@@ -7291,7 +7299,7 @@
         </is>
       </c>
       <c r="G122" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H122" s="4" t="inlineStr"/>
     </row>
@@ -7363,7 +7371,7 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H124" s="4" t="inlineStr"/>
     </row>
@@ -7399,7 +7407,7 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H125" s="4" t="inlineStr"/>
     </row>
@@ -7435,7 +7443,7 @@
         </is>
       </c>
       <c r="G126" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H126" s="4" t="inlineStr"/>
     </row>
@@ -7471,7 +7479,7 @@
         </is>
       </c>
       <c r="G127" s="4" t="n">
-        <v>0.16</v>
+        <v>0.05</v>
       </c>
       <c r="H127" s="4" t="inlineStr"/>
     </row>
@@ -7507,7 +7515,7 @@
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H128" s="4" t="inlineStr"/>
     </row>
@@ -7543,7 +7551,7 @@
         </is>
       </c>
       <c r="G129" s="4" t="n">
-        <v>1.28</v>
+        <v>1.06</v>
       </c>
       <c r="H129" s="4" t="inlineStr"/>
     </row>
@@ -7579,7 +7587,7 @@
         </is>
       </c>
       <c r="G130" s="4" t="n">
-        <v>1.19</v>
+        <v>0.67</v>
       </c>
       <c r="H130" s="4" t="inlineStr"/>
     </row>
@@ -7615,7 +7623,7 @@
         </is>
       </c>
       <c r="G131" s="4" t="n">
-        <v>2.45</v>
+        <v>1.6</v>
       </c>
       <c r="H131" s="4" t="inlineStr"/>
     </row>
@@ -7651,7 +7659,7 @@
         </is>
       </c>
       <c r="G132" s="4" t="n">
-        <v>2.03</v>
+        <v>1.54</v>
       </c>
       <c r="H132" s="4" t="inlineStr"/>
     </row>
@@ -7687,7 +7695,7 @@
         </is>
       </c>
       <c r="G133" s="4" t="n">
-        <v>2.4</v>
+        <v>1.91</v>
       </c>
       <c r="H133" s="4" t="inlineStr"/>
     </row>
@@ -7723,7 +7731,7 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>1.44</v>
+        <v>0.65</v>
       </c>
       <c r="H134" s="4" t="inlineStr"/>
     </row>
@@ -7759,7 +7767,7 @@
         </is>
       </c>
       <c r="G135" s="4" t="n">
-        <v>2.18</v>
+        <v>1.18</v>
       </c>
       <c r="H135" s="4" t="inlineStr"/>
     </row>
@@ -7795,7 +7803,7 @@
         </is>
       </c>
       <c r="G136" s="4" t="n">
-        <v>1.98</v>
+        <v>1.11</v>
       </c>
       <c r="H136" s="4" t="inlineStr"/>
     </row>
@@ -7831,7 +7839,7 @@
         </is>
       </c>
       <c r="G137" s="4" t="n">
-        <v>1.85</v>
+        <v>1.08</v>
       </c>
       <c r="H137" s="4" t="inlineStr"/>
     </row>
@@ -7867,7 +7875,7 @@
         </is>
       </c>
       <c r="G138" s="4" t="n">
-        <v>1.96</v>
+        <v>1.52</v>
       </c>
       <c r="H138" s="4" t="inlineStr"/>
     </row>
@@ -7903,7 +7911,7 @@
         </is>
       </c>
       <c r="G139" s="4" t="n">
-        <v>3.39</v>
+        <v>1.87</v>
       </c>
       <c r="H139" s="4" t="inlineStr"/>
     </row>
@@ -7939,7 +7947,7 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>1.25</v>
+        <v>0.58</v>
       </c>
       <c r="H140" s="4" t="inlineStr"/>
     </row>
@@ -7975,7 +7983,7 @@
         </is>
       </c>
       <c r="G141" s="4" t="n">
-        <v>1.32</v>
+        <v>0.65</v>
       </c>
       <c r="H141" s="4" t="inlineStr"/>
     </row>
@@ -8011,7 +8019,7 @@
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>1.14</v>
+        <v>0.46</v>
       </c>
       <c r="H142" s="4" t="inlineStr"/>
     </row>
@@ -8058,14 +8066,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Carga progresiva (10 → 25 → 50 → 100 usuarios). Cada usuario espera 1-3 s entre acciones. Resultados completos en docs/pruebas/estres/. La corrida en AWS se agrega al publicar.</t>
+          <t>Carga progresiva (10 → 25 → 50 → 100 usuarios). Cada usuario espera 1-3 s entre acciones. Resultados completos en docs/pruebas/estres/ (carpetas local/ y aws/).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Lectura: el cuello de botella es el inicio de sesión simultáneo (cada acceso calcula el hash PBKDF2 de la contraseña, ~0,3 s de CPU). Al subir 50-100 usuarios a razón de 10-20 por segundo, la CPU llega al 100 % mientras ingresan; una vez dentro, las páginas vuelven a responder en decenas de milisegundos. En la corrida local Locust compartía la misma CPU que el servidor.</t>
+          <t>Lectura: el cuello de botella es el inicio de sesión simultáneo (cada acceso calcula el hash PBKDF2 de la contraseña, ~0,3 s de CPU). Al subir 50-100 usuarios a razón de 10-20 por segundo, la CPU llega al 100 % mientras ingresan; una vez dentro, las páginas vuelven a responder en decenas de milisegundos. En la corrida local Locust compartía la misma CPU que el servidor; en AWS (t3.small) las latencias incluyen ~150 ms de red entre Chile y us-east-1. Mejora propuesta: más vCPU o un balanceador con dos instancias para absorber los ingresos simultáneos.</t>
         </is>
       </c>
     </row>
@@ -8159,7 +8167,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Local: 2 vCPU, 8 GB RAM, Ubuntu 24.04, Gunicorn 5 procesos × 2 hilos, MySQL 8.0 (Locust en la misma máquina)</t>
+          <t>AWS EC2 t3.small (2 vCPU, 2 GB RAM), us-east-1, Ubuntu 24.04, Nginx + Gunicorn (3 workers) + MySQL 8 local; Locust desde un equipo en Chile</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -8176,19 +8184,19 @@
         <v>10</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>382</v>
+        <v>477</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>6.5</v>
+        <v>5.3</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>33</v>
+        <v>244</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>46</v>
+        <v>320</v>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
@@ -8196,22 +8204,22 @@
         </is>
       </c>
       <c r="L5" s="4" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>360</v>
+        <v>4400</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>38</v>
+        <v>220</v>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>15 % / 77 %</t>
+          <t>13 % / 100 %</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>1292 MB (Gunicorn 400 MB · MySQL 434 MB)</t>
+          <t>949 MB (Gunicorn 217 MB · MySQL 418 MB)</t>
         </is>
       </c>
     </row>
@@ -8223,7 +8231,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Local: 2 vCPU, 8 GB RAM, Ubuntu 24.04, Gunicorn 5 procesos × 2 hilos, MySQL 8.0 (Locust en la misma máquina)</t>
+          <t>AWS EC2 t3.small (2 vCPU, 2 GB RAM), us-east-1, Ubuntu 24.04, Nginx + Gunicorn (3 workers) + MySQL 8 local; Locust desde un equipo en Chile</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -8240,19 +8248,19 @@
         <v>25</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>920</v>
+        <v>1094</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>15.6</v>
+        <v>12.2</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>44</v>
+        <v>516</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>63</v>
+        <v>3700</v>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
@@ -8260,22 +8268,22 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>90</v>
+        <v>4900</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>900</v>
+        <v>11000</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>26 % / 94 %</t>
+          <t>31 % / 100 %</t>
         </is>
       </c>
       <c r="P6" s="4" t="inlineStr">
         <is>
-          <t>1286 MB (Gunicorn 436 MB · MySQL 436 MB)</t>
+          <t>945 MB (Gunicorn 219 MB · MySQL 419 MB)</t>
         </is>
       </c>
     </row>
@@ -8287,7 +8295,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Local: 2 vCPU, 8 GB RAM, Ubuntu 24.04, Gunicorn 5 procesos × 2 hilos, MySQL 8.0 (Locust en la misma máquina)</t>
+          <t>AWS EC2 t3.small (2 vCPU, 2 GB RAM), us-east-1, Ubuntu 24.04, Nginx + Gunicorn (3 workers) + MySQL 8 local; Locust desde un equipo en Chile</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -8304,19 +8312,19 @@
         <v>50</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1718</v>
+        <v>1645</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>29.1</v>
+        <v>18.4</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>166</v>
+        <v>1175</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>1300</v>
+        <v>7100</v>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
@@ -8324,22 +8332,22 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>1600</v>
+        <v>2000</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>4000</v>
+        <v>31000</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>67</v>
+        <v>540</v>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>45 % / 100 %</t>
+          <t>59 % / 100 %</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>1261 MB (Gunicorn 441 MB · MySQL 437 MB)</t>
+          <t>940 MB (Gunicorn 223 MB · MySQL 420 MB)</t>
         </is>
       </c>
     </row>
@@ -8351,7 +8359,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Local: 2 vCPU, 8 GB RAM, Ubuntu 24.04, Gunicorn 5 procesos × 2 hilos, MySQL 8.0 (Locust en la misma máquina)</t>
+          <t>AWS EC2 t3.small (2 vCPU, 2 GB RAM), us-east-1, Ubuntu 24.04, Nginx + Gunicorn (3 workers) + MySQL 8 local; Locust desde un equipo en Chile</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -8368,19 +8376,19 @@
         <v>100</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>2921</v>
+        <v>1198</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>48.6</v>
+        <v>13.4</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>523</v>
+        <v>6097</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4300</v>
+        <v>38000</v>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
@@ -8388,22 +8396,22 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2400</v>
+        <v>43000</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>9900</v>
+        <v>53000</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>280</v>
+        <v>47000</v>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>76 % / 100 %</t>
+          <t>93 % / 100 %</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
         <is>
-          <t>1304 MB (Gunicorn 443 MB · MySQL 438 MB)</t>
+          <t>939 MB (Gunicorn 222 MB · MySQL 420 MB)</t>
         </is>
       </c>
     </row>
@@ -8502,7 +8510,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>10 usuarios: 50 · 25 usuarios: 90 · 50 usuarios: 1600 · 100 usuarios: 2400 (cumple hasta 25 usuarios)</t>
+          <t>10 usuarios: 700 · 25 usuarios: 4900 · 50 usuarios: 2000 · 100 usuarios: 43000 (cumple hasta 10 usuarios)</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -8524,12 +8532,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>10 usuarios: 360 · 25 usuarios: 900 · 50 usuarios: 4000 · 100 usuarios: 9900 (cumple hasta 25 usuarios)</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+          <t>10 usuarios: 4400 · 25 usuarios: 11000 · 50 usuarios: 31000 · 100 usuarios: 53000</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>No cumple</t>
         </is>
       </c>
     </row>
@@ -8546,12 +8554,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>10 usuarios: 38 · 25 usuarios: 110 · 50 usuarios: 67 · 100 usuarios: 280</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Cumple</t>
+          <t>10 usuarios: 220 · 25 usuarios: 210 · 50 usuarios: 540 · 100 usuarios: 47000 (cumple hasta 50 usuarios)</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Parcial</t>
         </is>
       </c>
     </row>
@@ -8568,7 +8576,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>10 usuarios: 32.6 · 25 usuarios: 44.2 · 50 usuarios: 166.1 · 100 usuarios: 522.7 (cumple hasta 50 usuarios)</t>
+          <t>10 usuarios: 243.7 · 25 usuarios: 516.3 · 50 usuarios: 1175.5 · 100 usuarios: 6097.5 (cumple hasta 10 usuarios)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -8590,12 +8598,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>10 usuarios: 15.2 · 25 usuarios: 26.3 · 50 usuarios: 44.8 · 100 usuarios: 76.4</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Cumple</t>
+          <t>10 usuarios: 13.4 · 25 usuarios: 31.2 · 50 usuarios: 58.7 · 100 usuarios: 93.0 (cumple hasta 50 usuarios)</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Parcial</t>
         </is>
       </c>
     </row>
@@ -8612,12 +8620,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Con 100 usuarios la mediana subió a 2300 ms durante el ingreso masivo (s 9) y volvió a 97 ms en el segundo 23 (14 s después), sin errores. · Al terminar la prueba: /salud/ 200 ({"estado": "ok"})</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Cumple</t>
+          <t>Con 100 usuarios la mediana no volvió a ≤ 100 ms durante la etapa. · Tras 10 usuarios: /salud/ 200 en 0.586003s · Tras 25 usuarios: /salud/ 200 en 0.272505s · Tras 50 usuarios: /salud/ 200 en 0.272486s · Tras 100 usuarios: /salud/ 200 en 0.272998s</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>No cumple</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EV2: envío real del código de recuperación por Gmail (SMTP)
- deploy/configurar_correo.sh: pide Gmail y contraseña de aplicación, los guarda solo en /opt/sgr/.env y envía un correo de prueba
- sgr_probar_correo: comando para verificar la configuración SMTP
- BandejaBackend: si el SMTP falla, registra el error y la recuperación continúa (copia en la bandeja)
- EMAIL_TIMEOUT de 15 s; prueba PR-22; matriz 139/139; README con los pasos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pruebas/matriz_pruebas_sgr_ev2.xlsx
+++ b/docs/pruebas/matriz_pruebas_sgr_ev2.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz funcional'!$A$4:$K$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pruebas automatizadas'!$A$4:$H$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pruebas automatizadas'!$A$4:$H$143</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Estrés'!$A$4:$P$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Umbrales'!$A$4:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Pendientes y simulados'!$A$4:$D$10</definedName>
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SGR La Serena · EV2 · 42 casos · 42 aprobados · base de datos de prueba: sqlite3 · generado 17-10-2026 12:02</t>
+          <t>SGR La Serena · EV2 · 42 casos · 42 aprobados · base de datos de prueba: sqlite3 · generado 17-10-2026 12:09</t>
         </is>
       </c>
     </row>
@@ -2986,7 +2986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H142"/>
+  <dimension ref="A1:H143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3009,7 +3009,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>138 pruebas · 138 aprobadas · comando: python manage.py test pruebas pruebas_ui</t>
+          <t>139 pruebas · 139 aprobadas · comando: python manage.py test pruebas pruebas_ui</t>
         </is>
       </c>
     </row>
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="G30" s="4" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
     </row>
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="G58" s="4" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="H58" s="4" t="inlineStr"/>
     </row>
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="G59" s="4" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="H59" s="4" t="inlineStr"/>
     </row>
@@ -5103,7 +5103,7 @@
         </is>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="H61" s="4" t="inlineStr"/>
     </row>
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="G62" s="4" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="H62" s="4" t="inlineStr"/>
     </row>
@@ -6111,7 +6111,7 @@
         </is>
       </c>
       <c r="G89" s="4" t="n">
-        <v>1.31</v>
+        <v>1.28</v>
       </c>
       <c r="H89" s="4" t="inlineStr"/>
     </row>
@@ -6478,27 +6478,27 @@
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>PS-01</t>
+          <t>PR-22</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>SweetAlert2</t>
+          <t>Recuperación</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Una operación exitosa se comunica a SweetAlert2 con nivel «success»</t>
+          <t>Si el servidor SMTP falla, la solicitud continúa y el código queda en la bandeja</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>pruebas/test_sistema.py</t>
+          <t>pruebas/test_recuperacion.py</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>test_exito_se_entrega_a_sweetalert</t>
+          <t>test_falla_smtp_no_interrumpe_recuperacion</t>
         </is>
       </c>
       <c r="F100" s="5" t="inlineStr">
@@ -6507,14 +6507,14 @@
         </is>
       </c>
       <c r="G100" s="4" t="n">
-        <v>0.01</v>
+        <v>2.02</v>
       </c>
       <c r="H100" s="4" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>PS-02</t>
+          <t>PS-01</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
@@ -6524,7 +6524,7 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Si la operación falla se muestra error y nunca un mensaje de éxito</t>
+          <t>Una operación exitosa se comunica a SweetAlert2 con nivel «success»</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
-          <t>test_error_no_muestra_exito</t>
+          <t>test_exito_se_entrega_a_sweetalert</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>PS-03</t>
+          <t>PS-02</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
@@ -6560,7 +6560,7 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Los formularios de eliminar y desactivar piden confirmación (data-confirmar)</t>
+          <t>Si la operación falla se muestra error y nunca un mensaje de éxito</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -6570,7 +6570,7 @@
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>test_confirmacion_antes_de_eliminar</t>
+          <t>test_error_no_muestra_exito</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
@@ -6586,7 +6586,7 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>PS-04</t>
+          <t>PS-03</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
@@ -6596,7 +6596,7 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>SweetAlert2 se sirve desde el propio sistema (sin depender de un CDN)</t>
+          <t>Los formularios de eliminar y desactivar piden confirmación (data-confirmar)</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -6606,7 +6606,7 @@
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
-          <t>test_libreria_cargada_localmente</t>
+          <t>test_confirmacion_antes_de_eliminar</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
@@ -6622,7 +6622,7 @@
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>PS-05</t>
+          <t>PS-04</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
@@ -6632,7 +6632,7 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Los mensajes con caracteres especiales no inyectan código</t>
+          <t>SweetAlert2 se sirve desde el propio sistema (sin depender de un CDN)</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -6642,7 +6642,7 @@
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>test_mensajes_escapados</t>
+          <t>test_libreria_cargada_localmente</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
@@ -6658,27 +6658,27 @@
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>PT-01</t>
+          <t>PS-05</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Ingreso de atención</t>
+          <t>SweetAlert2</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Registrar una atención entrega confirmación con identificador (folio)</t>
+          <t>Los mensajes con caracteres especiales no inyectan código</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>pruebas/test_atenciones.py</t>
+          <t>pruebas/test_sistema.py</t>
         </is>
       </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
-          <t>test_registro_correcto_con_folio</t>
+          <t>test_mensajes_escapados</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
@@ -6687,14 +6687,14 @@
         </is>
       </c>
       <c r="G105" s="4" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="H105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>PT-02</t>
+          <t>PT-01</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Delegación, responsable y fecha se asignan en el servidor, no desde el formulario</t>
+          <t>Registrar una atención entrega confirmación con identificador (folio)</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>test_delegacion_responsable_y_fecha_automaticos</t>
+          <t>test_registro_correcto_con_folio</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
@@ -6723,14 +6723,14 @@
         </is>
       </c>
       <c r="G106" s="4" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="H106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>PT-03</t>
+          <t>PT-02</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
@@ -6740,7 +6740,7 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Doble envío del mismo formulario no crea dos atenciones</t>
+          <t>Delegación, responsable y fecha se asignan en el servidor, no desde el formulario</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>test_doble_envio_no_duplica</t>
+          <t>test_delegacion_responsable_y_fecha_automaticos</t>
         </is>
       </c>
       <c r="F107" s="5" t="inlineStr">
@@ -6759,14 +6759,14 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="H107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>PT-04</t>
+          <t>PT-03</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
@@ -6776,7 +6776,7 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>La sub atención debe pertenecer al tipo elegido</t>
+          <t>Doble envío del mismo formulario no crea dos atenciones</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -6786,7 +6786,7 @@
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>test_sub_debe_pertenecer_al_tipo</t>
+          <t>test_doble_envio_no_duplica</t>
         </is>
       </c>
       <c r="F108" s="5" t="inlineStr">
@@ -6795,14 +6795,14 @@
         </is>
       </c>
       <c r="G108" s="4" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="H108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>PT-05</t>
+          <t>PT-04</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
@@ -6812,7 +6812,7 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Una sub atención inactiva no puede usarse</t>
+          <t>La sub atención debe pertenecer al tipo elegido</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -6822,7 +6822,7 @@
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
-          <t>test_sub_inactiva_rechazada</t>
+          <t>test_sub_debe_pertenecer_al_tipo</t>
         </is>
       </c>
       <c r="F109" s="5" t="inlineStr">
@@ -6838,7 +6838,7 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>PT-06</t>
+          <t>PT-05</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Un tipo de atención inactivo no puede usarse</t>
+          <t>Una sub atención inactiva no puede usarse</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -6858,7 +6858,7 @@
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>test_tipo_inactivo_rechazado</t>
+          <t>test_sub_inactiva_rechazada</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
@@ -6867,14 +6867,14 @@
         </is>
       </c>
       <c r="G110" s="4" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="H110" s="4" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>PT-07</t>
+          <t>PT-06</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
@@ -6884,7 +6884,7 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>El selector dependiente entrega solo sub atenciones activas del tipo</t>
+          <t>Un tipo de atención inactivo no puede usarse</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>test_api_subatenciones_solo_activas_del_tipo</t>
+          <t>test_tipo_inactivo_rechazado</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
@@ -6910,7 +6910,7 @@
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>PT-08</t>
+          <t>PT-07</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>El selector dependiente rechaza tipos inválidos o inactivos</t>
+          <t>El selector dependiente entrega solo sub atenciones activas del tipo</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -6930,7 +6930,7 @@
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>test_api_subatenciones_tipo_invalido</t>
+          <t>test_api_subatenciones_solo_activas_del_tipo</t>
         </is>
       </c>
       <c r="F112" s="5" t="inlineStr">
@@ -6946,7 +6946,7 @@
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>PT-09</t>
+          <t>PT-08</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
@@ -6956,7 +6956,7 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>Solicitante, tipo, sub atención y descripción son obligatorios</t>
+          <t>El selector dependiente rechaza tipos inválidos o inactivos</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -6966,7 +6966,7 @@
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
-          <t>test_campos_obligatorios</t>
+          <t>test_api_subatenciones_tipo_invalido</t>
         </is>
       </c>
       <c r="F113" s="5" t="inlineStr">
@@ -6982,7 +6982,7 @@
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>PT-10</t>
+          <t>PT-09</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>El RUT se valida con dígito verificador</t>
+          <t>Solicitante, tipo, sub atención y descripción son obligatorios</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>test_rut_invalido</t>
+          <t>test_campos_obligatorios</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
@@ -7018,7 +7018,7 @@
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>PT-11</t>
+          <t>PT-10</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>La descripción exige un mínimo de caracteres</t>
+          <t>El RUT se valida con dígito verificador</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
@@ -7038,7 +7038,7 @@
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
-          <t>test_descripcion_minima</t>
+          <t>test_rut_invalido</t>
         </is>
       </c>
       <c r="F115" s="5" t="inlineStr">
@@ -7047,14 +7047,14 @@
         </is>
       </c>
       <c r="G115" s="4" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="H115" s="4" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>PT-12</t>
+          <t>PT-11</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Un vecino ya registrado se reutiliza (sin duplicar por RUT)</t>
+          <t>La descripción exige un mínimo de caracteres</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>test_solicitante_existente_se_reutiliza</t>
+          <t>test_descripcion_minima</t>
         </is>
       </c>
       <c r="F116" s="5" t="inlineStr">
@@ -7090,7 +7090,7 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>PT-13</t>
+          <t>PT-12</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Abrir el formulario y salir (cancelar) no crea registros</t>
+          <t>Un vecino ya registrado se reutiliza (sin duplicar por RUT)</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>test_cancelar_no_crea</t>
+          <t>test_solicitante_existente_se_reutiliza</t>
         </is>
       </c>
       <c r="F117" s="5" t="inlineStr">
@@ -7119,14 +7119,14 @@
         </is>
       </c>
       <c r="G117" s="4" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="H117" s="4" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>PT-14</t>
+          <t>PT-13</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Un perfil sin permiso de crear no puede registrar atenciones</t>
+          <t>Abrir el formulario y salir (cancelar) no crea registros</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
@@ -7146,7 +7146,7 @@
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>test_sin_permiso_de_crear</t>
+          <t>test_cancelar_no_crea</t>
         </is>
       </c>
       <c r="F118" s="5" t="inlineStr">
@@ -7155,14 +7155,14 @@
         </is>
       </c>
       <c r="G118" s="4" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="H118" s="4" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>PT-15</t>
+          <t>PT-14</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
@@ -7172,7 +7172,7 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>El listado y el Excel de atenciones se limitan a la delegación activa</t>
+          <t>Un perfil sin permiso de crear no puede registrar atenciones</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
@@ -7182,7 +7182,7 @@
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>test_listado_solo_de_la_delegacion_activa</t>
+          <t>test_sin_permiso_de_crear</t>
         </is>
       </c>
       <c r="F119" s="5" t="inlineStr">
@@ -7191,14 +7191,14 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="H119" s="4" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>PT-16</t>
+          <t>PT-15</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
@@ -7208,7 +7208,7 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>La búsqueda de atenciones encuentra por folio y por RUT</t>
+          <t>El listado y el Excel de atenciones se limitan a la delegación activa</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>test_busqueda_por_folio_y_rut</t>
+          <t>test_listado_solo_de_la_delegacion_activa</t>
         </is>
       </c>
       <c r="F120" s="5" t="inlineStr">
@@ -7227,34 +7227,34 @@
         </is>
       </c>
       <c r="G120" s="4" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="H120" s="4" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>PU-01</t>
+          <t>PT-16</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Auditoría</t>
+          <t>Ingreso de atención</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>La auditoría nunca guarda contraseñas</t>
+          <t>La búsqueda de atenciones encuentra por folio y por RUT</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>pruebas/test_sistema.py</t>
+          <t>pruebas/test_atenciones.py</t>
         </is>
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
-          <t>test_auditoria_no_registra_contrasenas</t>
+          <t>test_busqueda_por_folio_y_rut</t>
         </is>
       </c>
       <c r="F121" s="5" t="inlineStr">
@@ -7263,14 +7263,14 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="H121" s="4" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>PU-02</t>
+          <t>PU-01</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>La auditoría lista y filtra eventos; no ofrece edición</t>
+          <t>La auditoría nunca guarda contraseñas</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>test_auditoria_solo_lectura_y_filtro</t>
+          <t>test_auditoria_no_registra_contrasenas</t>
         </is>
       </c>
       <c r="F122" s="5" t="inlineStr">
@@ -7306,17 +7306,17 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>PX-01</t>
+          <t>PU-02</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Auditoría</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>El punto de salud responde 200 con la base de datos disponible</t>
+          <t>La auditoría lista y filtra eventos; no ofrece edición</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
@@ -7326,7 +7326,7 @@
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>test_salud</t>
+          <t>test_auditoria_solo_lectura_y_filtro</t>
         </is>
       </c>
       <c r="F123" s="5" t="inlineStr">
@@ -7335,14 +7335,14 @@
         </is>
       </c>
       <c r="G123" s="4" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H123" s="4" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>PX-02</t>
+          <t>PX-01</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>Una ruta inexistente devuelve 404</t>
+          <t>El punto de salud responde 200 con la base de datos disponible</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
@@ -7362,7 +7362,7 @@
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>test_pagina_inexistente</t>
+          <t>test_salud</t>
         </is>
       </c>
       <c r="F124" s="5" t="inlineStr">
@@ -7371,14 +7371,14 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H124" s="4" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>PX-03</t>
+          <t>PX-02</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
@@ -7388,7 +7388,7 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Un registro inexistente devuelve 404 (no error 500)</t>
+          <t>Una ruta inexistente devuelve 404</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
@@ -7398,7 +7398,7 @@
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
-          <t>test_registro_inexistente</t>
+          <t>test_pagina_inexistente</t>
         </is>
       </c>
       <c r="F125" s="5" t="inlineStr">
@@ -7414,7 +7414,7 @@
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>PX-04</t>
+          <t>PX-03</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>Las respuestas incluyen cabeceras de seguridad básicas</t>
+          <t>Un registro inexistente devuelve 404 (no error 500)</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
@@ -7434,7 +7434,7 @@
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>test_cabeceras_de_seguridad</t>
+          <t>test_registro_inexistente</t>
         </is>
       </c>
       <c r="F126" s="5" t="inlineStr">
@@ -7443,14 +7443,14 @@
         </is>
       </c>
       <c r="G126" s="4" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H126" s="4" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>PX-05</t>
+          <t>PX-04</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>Los módulos en desarrollo son navegables y se identifican como simulados</t>
+          <t>Las respuestas incluyen cabeceras de seguridad básicas</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
@@ -7470,7 +7470,7 @@
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
-          <t>test_modulos_simulados_navegables</t>
+          <t>test_cabeceras_de_seguridad</t>
         </is>
       </c>
       <c r="F127" s="5" t="inlineStr">
@@ -7479,14 +7479,14 @@
         </is>
       </c>
       <c r="G127" s="4" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="H127" s="4" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>PX-06</t>
+          <t>PX-05</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
@@ -7496,7 +7496,7 @@
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>Un envío sin token CSRF se rechaza con una pantalla clara y sin guardar</t>
+          <t>Los módulos en desarrollo son navegables y se identifican como simulados</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
@@ -7506,7 +7506,7 @@
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>test_formulario_sin_token_csrf</t>
+          <t>test_modulos_simulados_navegables</t>
         </is>
       </c>
       <c r="F128" s="5" t="inlineStr">
@@ -7515,34 +7515,34 @@
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="H128" s="4" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>UI-01</t>
+          <t>PX-06</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>Interfaz (navegador)</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Acceso incorrecto muestra SweetAlert2 de error</t>
+          <t>Un envío sin token CSRF se rechaza con una pantalla clara y sin guardar</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>pruebas_ui/test_interfaz.py</t>
+          <t>pruebas/test_sistema.py</t>
         </is>
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
-          <t>test_ui01_error_de_acceso_con_sweetalert</t>
+          <t>test_formulario_sin_token_csrf</t>
         </is>
       </c>
       <c r="F129" s="5" t="inlineStr">
@@ -7551,14 +7551,14 @@
         </is>
       </c>
       <c r="G129" s="4" t="n">
-        <v>1.06</v>
+        <v>0</v>
       </c>
       <c r="H129" s="4" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>UI-02</t>
+          <t>UI-01</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Campos vacíos se marcan en el navegador antes de enviar</t>
+          <t>Acceso incorrecto muestra SweetAlert2 de error</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>test_ui02_validacion_en_navegador</t>
+          <t>test_ui01_error_de_acceso_con_sweetalert</t>
         </is>
       </c>
       <c r="F130" s="5" t="inlineStr">
@@ -7587,14 +7587,14 @@
         </is>
       </c>
       <c r="G130" s="4" t="n">
-        <v>0.67</v>
+        <v>1.06</v>
       </c>
       <c r="H130" s="4" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>UI-03</t>
+          <t>UI-02</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
@@ -7604,7 +7604,7 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Cancelar la confirmación de eliminar no elimina el registro</t>
+          <t>Campos vacíos se marcan en el navegador antes de enviar</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>test_ui03_cancelar_eliminacion_no_elimina</t>
+          <t>test_ui02_validacion_en_navegador</t>
         </is>
       </c>
       <c r="F131" s="5" t="inlineStr">
@@ -7623,14 +7623,14 @@
         </is>
       </c>
       <c r="G131" s="4" t="n">
-        <v>1.6</v>
+        <v>0.67</v>
       </c>
       <c r="H131" s="4" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>UI-04</t>
+          <t>UI-03</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Confirmar eliminar elimina y muestra éxito</t>
+          <t>Cancelar la confirmación de eliminar no elimina el registro</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
@@ -7650,7 +7650,7 @@
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>test_ui04_confirmar_eliminacion_y_mensaje_de_exito</t>
+          <t>test_ui03_cancelar_eliminacion_no_elimina</t>
         </is>
       </c>
       <c r="F132" s="5" t="inlineStr">
@@ -7659,14 +7659,14 @@
         </is>
       </c>
       <c r="G132" s="4" t="n">
-        <v>1.54</v>
+        <v>1.6</v>
       </c>
       <c r="H132" s="4" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>UI-05</t>
+          <t>UI-04</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
@@ -7676,7 +7676,7 @@
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Eliminar un registro con relaciones muestra error (no éxito)</t>
+          <t>Confirmar eliminar elimina y muestra éxito</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
-          <t>test_ui05_eliminacion_rechazada_muestra_error</t>
+          <t>test_ui04_confirmar_eliminacion_y_mensaje_de_exito</t>
         </is>
       </c>
       <c r="F133" s="5" t="inlineStr">
@@ -7695,14 +7695,14 @@
         </is>
       </c>
       <c r="G133" s="4" t="n">
-        <v>1.91</v>
+        <v>1.52</v>
       </c>
       <c r="H133" s="4" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>UI-06</t>
+          <t>UI-05</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Al cambiar el tipo, la sub atención se limpia y muestra solo las del tipo</t>
+          <t>Eliminar un registro con relaciones muestra error (no éxito)</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
@@ -7722,7 +7722,7 @@
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>test_ui06_lista_dependiente_y_limpieza</t>
+          <t>test_ui05_eliminacion_rechazada_muestra_error</t>
         </is>
       </c>
       <c r="F134" s="5" t="inlineStr">
@@ -7731,14 +7731,14 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>0.65</v>
+        <v>1.92</v>
       </c>
       <c r="H134" s="4" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>UI-07</t>
+          <t>UI-06</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
@@ -7748,7 +7748,7 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Doble clic en Guardar crea una sola atención y muestra el folio</t>
+          <t>Al cambiar el tipo, la sub atención se limpia y muestra solo las del tipo</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
-          <t>test_ui07_doble_envio_crea_una_sola_atencion</t>
+          <t>test_ui06_lista_dependiente_y_limpieza</t>
         </is>
       </c>
       <c r="F135" s="5" t="inlineStr">
@@ -7767,14 +7767,14 @@
         </is>
       </c>
       <c r="G135" s="4" t="n">
-        <v>1.18</v>
+        <v>0.98</v>
       </c>
       <c r="H135" s="4" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>UI-08</t>
+          <t>UI-07</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
@@ -7784,7 +7784,7 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Cancelar con cambios pide confirmación y no crea registros</t>
+          <t>Doble clic en Guardar crea una sola atención y muestra el folio</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
@@ -7794,7 +7794,7 @@
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>test_ui08_cancelar_formulario_con_cambios</t>
+          <t>test_ui07_doble_envio_crea_una_sola_atencion</t>
         </is>
       </c>
       <c r="F136" s="5" t="inlineStr">
@@ -7803,14 +7803,14 @@
         </is>
       </c>
       <c r="G136" s="4" t="n">
-        <v>1.11</v>
+        <v>1.13</v>
       </c>
       <c r="H136" s="4" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>UI-09</t>
+          <t>UI-08</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
@@ -7820,7 +7820,7 @@
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>Cambiar de delegación con cambios sin guardar muestra advertencia</t>
+          <t>Cancelar con cambios pide confirmación y no crea registros</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="E137" s="4" t="inlineStr">
         <is>
-          <t>test_ui09_cambio_de_delegacion_advierte_cambios</t>
+          <t>test_ui08_cancelar_formulario_con_cambios</t>
         </is>
       </c>
       <c r="F137" s="5" t="inlineStr">
@@ -7839,14 +7839,14 @@
         </is>
       </c>
       <c r="G137" s="4" t="n">
-        <v>1.08</v>
+        <v>1.11</v>
       </c>
       <c r="H137" s="4" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>UI-10</t>
+          <t>UI-09</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
@@ -7856,7 +7856,7 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>Confirmar el cambio de delegación actualiza cabecera y listado</t>
+          <t>Cambiar de delegación con cambios sin guardar muestra advertencia</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
@@ -7866,7 +7866,7 @@
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>test_ui10_cambio_de_delegacion_actualiza_cabecera</t>
+          <t>test_ui09_cambio_de_delegacion_advierte_cambios</t>
         </is>
       </c>
       <c r="F138" s="5" t="inlineStr">
@@ -7875,14 +7875,14 @@
         </is>
       </c>
       <c r="G138" s="4" t="n">
-        <v>1.52</v>
+        <v>1.09</v>
       </c>
       <c r="H138" s="4" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>UI-11</t>
+          <t>UI-10</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Cada perfil ve solo los menús autorizados</t>
+          <t>Confirmar el cambio de delegación actualiza cabecera y listado</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
@@ -7902,7 +7902,7 @@
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
-          <t>test_ui11_menu_por_perfil</t>
+          <t>test_ui10_cambio_de_delegacion_actualiza_cabecera</t>
         </is>
       </c>
       <c r="F139" s="5" t="inlineStr">
@@ -7911,14 +7911,14 @@
         </is>
       </c>
       <c r="G139" s="4" t="n">
-        <v>1.87</v>
+        <v>0.71</v>
       </c>
       <c r="H139" s="4" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>UI-12</t>
+          <t>UI-11</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
@@ -7928,7 +7928,7 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Recuperación: pegar el código llena las 6 casillas y el reenvío espera 45 s</t>
+          <t>Cada perfil ve solo los menús autorizados</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
@@ -7938,7 +7938,7 @@
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>test_ui12_recuperacion_casillas_y_cuenta_regresiva</t>
+          <t>test_ui11_menu_por_perfil</t>
         </is>
       </c>
       <c r="F140" s="5" t="inlineStr">
@@ -7947,14 +7947,14 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>0.58</v>
+        <v>1.88</v>
       </c>
       <c r="H140" s="4" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>UI-13</t>
+          <t>UI-12</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Exportar a Excel descarga un .xlsx con los filtros aplicados</t>
+          <t>Recuperación: pegar el código llena las 6 casillas y el reenvío espera 45 s</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
@@ -7974,7 +7974,7 @@
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
-          <t>test_ui13_exportar_descarga_excel</t>
+          <t>test_ui12_recuperacion_casillas_y_cuenta_regresiva</t>
         </is>
       </c>
       <c r="F141" s="5" t="inlineStr">
@@ -7983,48 +7983,84 @@
         </is>
       </c>
       <c r="G141" s="4" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="H141" s="4" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
+          <t>UI-13</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>Interfaz (navegador)</t>
+        </is>
+      </c>
+      <c r="C142" s="4" t="inlineStr">
+        <is>
+          <t>Exportar a Excel descarga un .xlsx con los filtros aplicados</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>pruebas_ui/test_interfaz.py</t>
+        </is>
+      </c>
+      <c r="E142" s="4" t="inlineStr">
+        <is>
+          <t>test_ui13_exportar_descarga_excel</t>
+        </is>
+      </c>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="G142" s="4" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="H142" s="4" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="inlineStr">
+        <is>
           <t>UI-14</t>
         </is>
       </c>
-      <c r="B142" s="4" t="inlineStr">
+      <c r="B143" s="4" t="inlineStr">
         <is>
           <t>Interfaz (navegador)</t>
         </is>
       </c>
-      <c r="C142" s="4" t="inlineStr">
+      <c r="C143" s="4" t="inlineStr">
         <is>
           <t>En pantalla de teléfono el menú se abre con el botón y la cabecera se mantiene</t>
         </is>
       </c>
-      <c r="D142" s="4" t="inlineStr">
+      <c r="D143" s="4" t="inlineStr">
         <is>
           <t>pruebas_ui/test_interfaz.py</t>
         </is>
       </c>
-      <c r="E142" s="4" t="inlineStr">
+      <c r="E143" s="4" t="inlineStr">
         <is>
           <t>test_ui14_vista_movil</t>
         </is>
       </c>
-      <c r="F142" s="5" t="inlineStr">
-        <is>
-          <t>Aprobada</t>
-        </is>
-      </c>
-      <c r="G142" s="4" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="H142" s="4" t="inlineStr"/>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="G143" s="4" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="H143" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H142"/>
+  <autoFilter ref="A4:H143"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>